<commit_message>
spotted issues with Nationality and Age in ITRA TXT file so updated code and TXT file
</commit_message>
<xml_diff>
--- a/TOR330 Data/4. TOR330 Timetable Data/TOR330 - Timetable.xlsx
+++ b/TOR330 Data/4. TOR330 Timetable Data/TOR330 - Timetable.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karina\Portfolio\Tor_Des_Geants\TOR330 Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Karina\Portfolio\TORX\TOR330 Data\4. TOR330 Timetable Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{887376AB-A46D-44E4-BDEC-4B97EBDD4BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFBFC421-6658-4949-A997-29E2229C7040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TOR330 Timetable 2023" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet4" sheetId="5" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="3" r:id="rId4"/>
+    <sheet name="Sheet3" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,14 +33,14 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="hMaWvR4Q+WTNWHq23wGtHonHnOLu5M+4GjW8/EVtmCI="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="hMaWvR4Q+WTNWHq23wGtHonHnOLu5M+4GjW8/EVtmCI="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="377">
   <si>
     <r>
       <rPr>
@@ -1456,17 +1459,21 @@
   <si>
     <t>Wave 2 Cut off time</t>
   </si>
+  <si>
+    <t>Tme Between Cut Offs</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0_-;\-* #,##0_-;_-* \-??_-;_-@"/>
+    <numFmt numFmtId="168" formatCode="[$-F400]h:mm:ss\ am/pm"/>
   </numFmts>
-  <fonts count="26">
+  <fonts count="27">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1617,8 +1624,15 @@
       <color theme="1"/>
       <name val="Helvetica Neue"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1709,8 +1723,14 @@
         <bgColor rgb="FFD9EAD3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1718,11 +1738,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1941,10 +1970,25 @@
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1954,9 +1998,6 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1966,15 +2007,30 @@
     <xf numFmtId="49" fontId="7" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="168" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2204,23 +2260,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="6" customHeight="1">
-      <c r="A1" s="76"/>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="75"/>
-      <c r="L1" s="75"/>
-      <c r="M1" s="75"/>
-      <c r="N1" s="75"/>
-      <c r="O1" s="75"/>
-      <c r="P1" s="75"/>
-      <c r="Q1" s="75"/>
+      <c r="A1" s="81"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="76"/>
+      <c r="N1" s="76"/>
+      <c r="O1" s="76"/>
+      <c r="P1" s="76"/>
+      <c r="Q1" s="76"/>
     </row>
     <row r="2" spans="1:17" ht="46.5" customHeight="1">
       <c r="A2" s="1"/>
@@ -2287,135 +2343,135 @@
       </c>
     </row>
     <row r="4" spans="1:17" ht="6" customHeight="1">
-      <c r="A4" s="77"/>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="75"/>
-      <c r="I4" s="75"/>
-      <c r="J4" s="75"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="75"/>
-      <c r="M4" s="75"/>
-      <c r="N4" s="75"/>
-      <c r="O4" s="75"/>
-      <c r="P4" s="75"/>
-      <c r="Q4" s="75"/>
+      <c r="A4" s="82"/>
+      <c r="B4" s="76"/>
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="76"/>
+      <c r="Q4" s="76"/>
     </row>
     <row r="5" spans="1:17" ht="84.75" customHeight="1">
-      <c r="A5" s="78" t="s">
+      <c r="A5" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="75"/>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75"/>
-      <c r="E5" s="75"/>
-      <c r="F5" s="75"/>
-      <c r="G5" s="75"/>
-      <c r="H5" s="75"/>
-      <c r="I5" s="75"/>
-      <c r="J5" s="75"/>
-      <c r="K5" s="75"/>
-      <c r="L5" s="75"/>
-      <c r="M5" s="75"/>
-      <c r="N5" s="75"/>
-      <c r="O5" s="75"/>
-      <c r="P5" s="75"/>
-      <c r="Q5" s="75"/>
+      <c r="B5" s="76"/>
+      <c r="C5" s="76"/>
+      <c r="D5" s="76"/>
+      <c r="E5" s="76"/>
+      <c r="F5" s="76"/>
+      <c r="G5" s="76"/>
+      <c r="H5" s="76"/>
+      <c r="I5" s="76"/>
+      <c r="J5" s="76"/>
+      <c r="K5" s="76"/>
+      <c r="L5" s="76"/>
+      <c r="M5" s="76"/>
+      <c r="N5" s="76"/>
+      <c r="O5" s="76"/>
+      <c r="P5" s="76"/>
+      <c r="Q5" s="76"/>
     </row>
     <row r="6" spans="1:17" ht="24.75" customHeight="1">
-      <c r="A6" s="79" t="s">
+      <c r="A6" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="80" t="s">
+      <c r="B6" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="79" t="s">
+      <c r="C6" s="77" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="79" t="s">
+      <c r="D6" s="77" t="s">
         <v>22</v>
       </c>
-      <c r="E6" s="83" t="s">
+      <c r="E6" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="79" t="s">
+      <c r="F6" s="77" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="79" t="s">
+      <c r="G6" s="77" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="84" t="s">
+      <c r="H6" s="78" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="85"/>
-      <c r="J6" s="81" t="s">
+      <c r="I6" s="79"/>
+      <c r="J6" s="85" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="75"/>
-      <c r="L6" s="75"/>
-      <c r="M6" s="75"/>
-      <c r="N6" s="82" t="s">
+      <c r="K6" s="76"/>
+      <c r="L6" s="76"/>
+      <c r="M6" s="76"/>
+      <c r="N6" s="86" t="s">
         <v>28</v>
       </c>
-      <c r="O6" s="75"/>
-      <c r="P6" s="75"/>
-      <c r="Q6" s="75"/>
+      <c r="O6" s="76"/>
+      <c r="P6" s="76"/>
+      <c r="Q6" s="76"/>
     </row>
     <row r="7" spans="1:17" ht="25.5" customHeight="1">
-      <c r="A7" s="75"/>
-      <c r="B7" s="75"/>
-      <c r="C7" s="75"/>
-      <c r="D7" s="75"/>
-      <c r="E7" s="75"/>
-      <c r="F7" s="75"/>
-      <c r="G7" s="75"/>
-      <c r="H7" s="75"/>
-      <c r="I7" s="75"/>
-      <c r="J7" s="81" t="s">
+      <c r="A7" s="76"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
+      <c r="F7" s="76"/>
+      <c r="G7" s="76"/>
+      <c r="H7" s="76"/>
+      <c r="I7" s="76"/>
+      <c r="J7" s="85" t="s">
         <v>29</v>
       </c>
-      <c r="K7" s="81" t="s">
+      <c r="K7" s="85" t="s">
         <v>30</v>
       </c>
-      <c r="L7" s="81" t="s">
+      <c r="L7" s="85" t="s">
         <v>31</v>
       </c>
-      <c r="M7" s="75"/>
-      <c r="N7" s="82" t="s">
+      <c r="M7" s="76"/>
+      <c r="N7" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="O7" s="82" t="s">
+      <c r="O7" s="86" t="s">
         <v>30</v>
       </c>
-      <c r="P7" s="82" t="s">
+      <c r="P7" s="86" t="s">
         <v>31</v>
       </c>
-      <c r="Q7" s="75"/>
+      <c r="Q7" s="76"/>
     </row>
     <row r="8" spans="1:17" ht="21" customHeight="1">
-      <c r="A8" s="75"/>
-      <c r="B8" s="75"/>
-      <c r="C8" s="75"/>
-      <c r="D8" s="75"/>
-      <c r="E8" s="75"/>
-      <c r="F8" s="75"/>
-      <c r="G8" s="75"/>
-      <c r="H8" s="75"/>
-      <c r="I8" s="75"/>
-      <c r="J8" s="75"/>
-      <c r="K8" s="75"/>
+      <c r="A8" s="76"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
+      <c r="F8" s="76"/>
+      <c r="G8" s="76"/>
+      <c r="H8" s="76"/>
+      <c r="I8" s="76"/>
+      <c r="J8" s="76"/>
+      <c r="K8" s="76"/>
       <c r="L8" s="13" t="s">
         <v>32</v>
       </c>
       <c r="M8" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="N8" s="75"/>
-      <c r="O8" s="75"/>
+      <c r="N8" s="76"/>
+      <c r="O8" s="76"/>
       <c r="P8" s="14" t="s">
         <v>32</v>
       </c>
@@ -5693,25 +5749,25 @@
       <c r="O89" s="68"/>
     </row>
     <row r="90" spans="1:17" ht="15.75" customHeight="1">
-      <c r="A90" s="74" t="s">
+      <c r="A90" s="80" t="s">
         <v>334</v>
       </c>
-      <c r="B90" s="75"/>
-      <c r="C90" s="75"/>
-      <c r="D90" s="75"/>
-      <c r="E90" s="75"/>
-      <c r="F90" s="75"/>
-      <c r="G90" s="75"/>
-      <c r="H90" s="75"/>
-      <c r="I90" s="75"/>
-      <c r="J90" s="75"/>
-      <c r="K90" s="75"/>
-      <c r="L90" s="75"/>
-      <c r="M90" s="75"/>
-      <c r="N90" s="75"/>
-      <c r="O90" s="75"/>
-      <c r="P90" s="75"/>
-      <c r="Q90" s="75"/>
+      <c r="B90" s="76"/>
+      <c r="C90" s="76"/>
+      <c r="D90" s="76"/>
+      <c r="E90" s="76"/>
+      <c r="F90" s="76"/>
+      <c r="G90" s="76"/>
+      <c r="H90" s="76"/>
+      <c r="I90" s="76"/>
+      <c r="J90" s="76"/>
+      <c r="K90" s="76"/>
+      <c r="L90" s="76"/>
+      <c r="M90" s="76"/>
+      <c r="N90" s="76"/>
+      <c r="O90" s="76"/>
+      <c r="P90" s="76"/>
+      <c r="Q90" s="76"/>
     </row>
     <row r="91" spans="1:17" ht="15.75" customHeight="1">
       <c r="A91" s="68"/>
@@ -5800,11 +5856,6 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="F6:F8"/>
-    <mergeCell ref="G6:G8"/>
-    <mergeCell ref="H6:H8"/>
-    <mergeCell ref="I6:I8"/>
     <mergeCell ref="A90:Q90"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A4:Q4"/>
@@ -5821,6 +5872,11 @@
     <mergeCell ref="N7:N8"/>
     <mergeCell ref="O7:O8"/>
     <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="F6:F8"/>
+    <mergeCell ref="G6:G8"/>
+    <mergeCell ref="H6:H8"/>
+    <mergeCell ref="I6:I8"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.25" right="0.25" top="0.19685039370078738" bottom="0.19685039370078738" header="0" footer="0"/>
@@ -7664,4 +7720,562 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5BAD15C-6AAC-4EB7-89F5-584238B0F870}">
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="2" max="2" width="21.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="94"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="94"/>
+    </row>
+    <row r="2" spans="1:6" ht="39" thickBot="1">
+      <c r="A2" s="94"/>
+      <c r="B2" s="87" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="88" t="s">
+        <v>374</v>
+      </c>
+      <c r="D2" s="89" t="s">
+        <v>375</v>
+      </c>
+      <c r="E2" s="93" t="s">
+        <v>376</v>
+      </c>
+      <c r="F2" s="94"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="94"/>
+      <c r="B3" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="90"/>
+      <c r="F3" s="94"/>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="94"/>
+      <c r="B4" s="37" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="91">
+        <v>0.22916666667151731</v>
+      </c>
+      <c r="F4" s="94"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="94"/>
+      <c r="B5" s="47" t="s">
+        <v>335</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="92">
+        <v>0.5625</v>
+      </c>
+      <c r="F5" s="94"/>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="94"/>
+      <c r="B6" s="47" t="s">
+        <v>336</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="E6" s="92">
+        <v>8.3333333328482695E-2</v>
+      </c>
+      <c r="F6" s="94"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="94"/>
+      <c r="B7" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="E7" s="91">
+        <v>0.52083333333575865</v>
+      </c>
+      <c r="F7" s="94"/>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="94"/>
+      <c r="B8" s="47" t="s">
+        <v>340</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="E8" s="92">
+        <v>0.35416666666424135</v>
+      </c>
+      <c r="F8" s="94"/>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="94"/>
+      <c r="B9" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" s="92">
+        <v>8.3333333335758653E-2</v>
+      </c>
+      <c r="F9" s="94"/>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="94"/>
+      <c r="B10" s="47" t="s">
+        <v>344</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="E10" s="92">
+        <v>0.75</v>
+      </c>
+      <c r="F10" s="94"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="94"/>
+      <c r="B11" s="47" t="s">
+        <v>345</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>147</v>
+      </c>
+      <c r="E11" s="92">
+        <v>8.3333333335758653E-2</v>
+      </c>
+      <c r="F11" s="94"/>
+    </row>
+    <row r="12" spans="1:6" ht="24">
+      <c r="A12" s="94"/>
+      <c r="B12" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="E12" s="91">
+        <v>0.45833333332848269</v>
+      </c>
+      <c r="F12" s="94"/>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="94"/>
+      <c r="B13" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="E13" s="91">
+        <v>0.27083333333333331</v>
+      </c>
+      <c r="F13" s="94"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="94"/>
+      <c r="B14" s="47" t="s">
+        <v>352</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="E14" s="92">
+        <v>0.14583333333575865</v>
+      </c>
+      <c r="F14" s="94"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="94"/>
+      <c r="B15" s="47" t="s">
+        <v>353</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>202</v>
+      </c>
+      <c r="E15" s="92">
+        <v>8.3333333328482695E-2</v>
+      </c>
+      <c r="F15" s="94"/>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="94"/>
+      <c r="B16" s="37" t="s">
+        <v>210</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>213</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="E16" s="91">
+        <v>0.5</v>
+      </c>
+      <c r="F16" s="94"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="94"/>
+      <c r="B17" s="47" t="s">
+        <v>355</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="D17" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="E17" s="92">
+        <v>0.25</v>
+      </c>
+      <c r="F17" s="94"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="94"/>
+      <c r="B18" s="47" t="s">
+        <v>356</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="D18" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="E18" s="92">
+        <v>8.3333333335758653E-2</v>
+      </c>
+      <c r="F18" s="94"/>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="94"/>
+      <c r="B19" s="37" t="s">
+        <v>263</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="D19" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="E19" s="91">
+        <v>0.625</v>
+      </c>
+      <c r="F19" s="94"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="94"/>
+      <c r="B20" s="47" t="s">
+        <v>364</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="E20" s="92">
+        <v>0.20833333333575865</v>
+      </c>
+      <c r="F20" s="94"/>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="94"/>
+      <c r="B21" s="47" t="s">
+        <v>365</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D21" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="E21" s="92">
+        <v>8.3333333328482695E-2</v>
+      </c>
+      <c r="F21" s="94"/>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="94"/>
+      <c r="B22" s="47" t="s">
+        <v>327</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="D22" s="14" t="s">
+        <v>333</v>
+      </c>
+      <c r="E22" s="92">
+        <v>0.875</v>
+      </c>
+      <c r="F22" s="94"/>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="94"/>
+      <c r="B23" s="96"/>
+      <c r="C23" s="96"/>
+      <c r="D23" s="96"/>
+      <c r="E23" s="96"/>
+      <c r="F23" s="94"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="96"/>
+      <c r="B24" s="96"/>
+      <c r="C24" s="96"/>
+      <c r="D24" s="96"/>
+      <c r="E24" s="96"/>
+      <c r="F24" s="96"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08373683-E0AE-4F05-96DF-6622E5D8A64B}">
+  <dimension ref="B2:D16"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="2" max="2" width="25.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4" ht="38.25">
+      <c r="B2" s="74" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>374</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4">
+      <c r="B3" s="70" t="s">
+        <v>372</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4">
+      <c r="B4" s="47" t="s">
+        <v>335</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4">
+      <c r="B5" s="47" t="s">
+        <v>336</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="B6" s="47" t="s">
+        <v>340</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="B7" s="47" t="s">
+        <v>341</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4">
+      <c r="B8" s="47" t="s">
+        <v>344</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="B9" s="47" t="s">
+        <v>345</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4">
+      <c r="B10" s="47" t="s">
+        <v>352</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4">
+      <c r="B11" s="47" t="s">
+        <v>353</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="D11" s="14" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4">
+      <c r="B12" s="47" t="s">
+        <v>355</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>229</v>
+      </c>
+      <c r="D12" s="14" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="13" spans="2:4">
+      <c r="B13" s="47" t="s">
+        <v>356</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="D13" s="14" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="14" spans="2:4">
+      <c r="B14" s="47" t="s">
+        <v>364</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>285</v>
+      </c>
+      <c r="D14" s="14" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4">
+      <c r="B15" s="47" t="s">
+        <v>365</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="D15" s="14" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4">
+      <c r="B16" s="47" t="s">
+        <v>327</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>331</v>
+      </c>
+      <c r="D16" s="14" t="s">
+        <v>333</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813A0E10-8EC7-405B-95EC-4EDDBA3E7A80}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>